<commit_message>
Update imageTrend images and spreadsheet
Replace binary assets in imageTrend: updated 01.jpg and 02.jpg, and an updated Excel spreadsheet (non-ASCII filename). These are asset updates (binary diffs) to refresh imagery and associated data in the imageTrend directory.
</commit_message>
<xml_diff>
--- a/画像生成.xlsx
+++ b/画像生成.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freecar\Documents\noutore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA3A0D6-2225-4A75-A6F2-6030D50F95AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D14B8C7-F4A2-4CE8-BB17-64B719E06104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="15326" windowWidth="24892" windowHeight="14914" xr2:uid="{3F2C732E-DC39-48C4-929C-44CCFEC2600E}"/>
   </bookViews>
@@ -57,7 +57,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1"/>
+  </si>
   <si>
     <t xml:space="preserve"> </t>
     <phoneticPr fontId="1"/>
@@ -306,7 +310,7 @@
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>クロード・ミュトス</a:t>
+            <a:t>ポテトチップス</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="2000">
             <a:solidFill>
@@ -1802,22 +1806,15 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1600">
+            <a:rPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1800" b="1">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>スマホ農場</a:t>
+            <a:t>BeReal</a:t>
           </a:r>
-          <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1600">
-            <a:solidFill>
-              <a:schemeClr val="bg1"/>
-            </a:solidFill>
-            <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
-          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -4299,13 +4296,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{596861FA-685D-46AF-8AC4-FE498235E344}">
-  <dimension ref="E2"/>
+  <dimension ref="B1:E2"/>
   <sheetFormatPr defaultRowHeight="90" customHeight="1" x14ac:dyDescent="0.65"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="5:5" ht="90" customHeight="1" x14ac:dyDescent="0.65">
+    <row r="1" spans="2:5" ht="90" customHeight="1" x14ac:dyDescent="0.65">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" ht="90" customHeight="1" x14ac:dyDescent="0.65">
       <c r="E2" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Update images and generation spreadsheet
Update trend images (01.jpg, 02.jpg) and image generation spreadsheet. Remove temporary Excel lock file.
</commit_message>
<xml_diff>
--- a/画像生成.xlsx
+++ b/画像生成.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freecar\Documents\noutore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81010572-8800-460F-BFD5-16E24A293CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84050F98-7077-41B1-85CE-C99ADAFF9006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="15326" windowWidth="24892" windowHeight="15634" xr2:uid="{3F2C732E-DC39-48C4-929C-44CCFEC2600E}"/>
   </bookViews>
@@ -306,7 +306,7 @@
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>スターリンク</a:t>
+            <a:t>推し活</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="2000">
             <a:solidFill>
@@ -1809,7 +1809,7 @@
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>ポテトチップス</a:t>
+            <a:t>蚊</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1800" b="1">
             <a:solidFill>

</xml_diff>

<commit_message>
Update trend images and spreadsheet
Updated imageTrend/01.jpg and imageTrend/02.jpg along with the 画像生成.xlsx data file. Removed temporary Excel lock file.
</commit_message>
<xml_diff>
--- a/画像生成.xlsx
+++ b/画像生成.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freecar\Documents\noutore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84050F98-7077-41B1-85CE-C99ADAFF9006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB33C33-C665-47E2-B807-DFE40FAD61C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="15326" windowWidth="24892" windowHeight="15634" xr2:uid="{3F2C732E-DC39-48C4-929C-44CCFEC2600E}"/>
   </bookViews>
@@ -306,7 +306,7 @@
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>推し活</a:t>
+            <a:t>ハンディファン</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="2000">
             <a:solidFill>
@@ -1809,7 +1809,7 @@
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>蚊</a:t>
+            <a:t>ドパ人</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1800" b="1">
             <a:solidFill>

</xml_diff>

<commit_message>
Update imageTrend images and Excel file
Replace imageTrend/01.jpg and imageTrend/02.jpg with updated binaries and update the Excel file in imageTrend (filename encoded in UTF-8). No source code changes.
</commit_message>
<xml_diff>
--- a/画像生成.xlsx
+++ b/画像生成.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freecar\Documents\noutore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB33C33-C665-47E2-B807-DFE40FAD61C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE2B518-01B6-452F-A438-E91802B3D6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="15326" windowWidth="24892" windowHeight="15634" xr2:uid="{3F2C732E-DC39-48C4-929C-44CCFEC2600E}"/>
   </bookViews>
@@ -299,14 +299,24 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="2000">
+            <a:rPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="2000">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>ハンディファン</a:t>
+            <a:t>AI</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="2000" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
+            </a:rPr>
+            <a:t>ハック</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="2000">
             <a:solidFill>
@@ -1802,22 +1812,15 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="1800" b="1">
+            <a:rPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1800" b="1">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>ドパ人</a:t>
+            <a:t>00000JAPAN</a:t>
           </a:r>
-          <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1800" b="1">
-            <a:solidFill>
-              <a:schemeClr val="bg1"/>
-            </a:solidFill>
-            <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
-          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>

</xml_diff>

<commit_message>
Refresh image trend assets
Updated the image trend JPGs and the associated Excel workbook to reflect the latest generated data and visuals.
</commit_message>
<xml_diff>
--- a/画像生成.xlsx
+++ b/画像生成.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freecar\Documents\noutore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7241F6AD-28EA-49A5-A319-AAD64DA11615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05EB9100-2234-4308-B762-B71140CE66E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="15326" windowWidth="24892" windowHeight="15634" xr2:uid="{3F2C732E-DC39-48C4-929C-44CCFEC2600E}"/>
   </bookViews>
@@ -310,7 +310,7 @@
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>サンブロック</a:t>
+            <a:t>ほんだし</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="2000">
             <a:solidFill>
@@ -1813,7 +1813,7 @@
               <a:latin typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
               <a:ea typeface="HGP創英角ｺﾞｼｯｸUB" panose="020B0900000000000000" pitchFamily="50" charset="-128"/>
             </a:rPr>
-            <a:t>モジョジョジョ</a:t>
+            <a:t>ちいかわ</a:t>
           </a:r>
           <a:endParaRPr kumimoji="1" lang="en-US" altLang="ja-JP" sz="1800" b="1">
             <a:solidFill>

</xml_diff>